<commit_message>
Implement V1.2 workflows and align platform extract contracts
</commit_message>
<xml_diff>
--- a/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
+++ b/platform-data-collection/v1.1-extract/analytic-registry-v1.1-extract.xlsx
@@ -2,23 +2,23 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R35e06569631d4547"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R02d97914bffd4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="Rdfd902765592404b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R306371199fef4693"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R0ff78ae54c4147ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R746ebc82870e40ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R695faf2619634fb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="R4a4d6630eb8a4967"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="R32fc44687fd641ff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R2794a9d89628442e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="Re0c316331b194d64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R21201718dbd34235"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="Re1dc4cb9718f44d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R02803f40f78248bd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R27ef375b836d411c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Re42b7c9b960043d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="Raa76edd8102b4f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R706ca3e3cead41ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Column_Dictionary" sheetId="2" r:id="R28034bfd27a34b2b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Migration_Map" sheetId="3" r:id="R518a544153a94679"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Run_Context" sheetId="4" r:id="R280a5550c7354108"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage" sheetId="5" r:id="R7c779a88de96474a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspaces" sheetId="6" r:id="R98609a8e68a54661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="7" r:id="R10e17fd14ff94057"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Workspace_Assets" sheetId="8" r:id="Rf8ac10d2bd6e4a32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Connections" sheetId="9" r:id="Rcf5163258ade4a8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Connections" sheetId="10" r:id="R02c2dc5c4b084c02"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Asset_Dependencies" sheetId="11" r:id="R9e0d9ade00a84c4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Platform_Users" sheetId="12" r:id="R597e2a774d2e4fe4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Directory_Users" sheetId="13" r:id="R648dd15adf76471b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Object_Users" sheetId="14" r:id="R1ea91791cd074426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tableau_Output" sheetId="15" r:id="R8c03e708b9bb4834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PowerBI_Output" sheetId="16" r:id="Rae4e244ce4c74961"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alteryx_Output" sheetId="17" r:id="R8a8e4ff0505f4409"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -758,7 +758,7 @@
         <x:v>2. Declare coverage</x:v>
       </x:c>
       <x:c r="B9" s="17" t="str">
-        <x:v>Provide one Coverage row for each dataset in the agreed scope. Distinguish Complete, Partial, NotCollected, and Failed. Empty input does not prove absence.</x:v>
+        <x:v>Provide one Coverage row per dataset. Complete and Partial require exact delivered row counts. Failed and NotCollected require NULL counts and no data rows. Empty input does not prove absence.</x:v>
       </x:c>
       <x:c r="C9" s="17" t="str">
         <x:v>Coverage</x:v>
@@ -777,15 +777,15 @@
       </x:c>
       <x:c r="D10" s="4" t="str"/>
     </x:row>
-    <x:row r="11" ht="36" customHeight="1">
+    <x:row r="11" ht="47.25" customHeight="1">
       <x:c r="A11" s="17" t="str">
-        <x:v>4. Validate and load</x:v>
+        <x:v>4. Validate and accept</x:v>
       </x:c>
       <x:c r="B11" s="17" t="str">
-        <x:v>Ignore only fully blank template rows. Quarantine invalid nonblank rows. Validate keys, references, and coverage before manual SQL Server staging.</x:v>
+        <x:v>Stage all nonblank records for validation. Structural errors block the whole delivery. The registry operator accepts valid deliveries, including Partial coverage and unresolved references. Assign unresolved cases to Platform Manager; preserve original evidence dates.</x:v>
       </x:c>
       <x:c r="C11" s="17" t="str">
-        <x:v>Platform Manager</x:v>
+        <x:v>Registry operator</x:v>
       </x:c>
       <x:c r="D11" s="17" t="str"/>
     </x:row>
@@ -806,7 +806,7 @@
         <x:v>Refresh identity</x:v>
       </x:c>
       <x:c r="B13" s="17" t="str">
-        <x:v>Resolve native objects within PlatformCode, PlatformInstanceKey, NativeScopeKey, native object type, and native ID. Names remain display fields.</x:v>
+        <x:v>Resolve objects by platform, instance, native scope, entity kind, and native ID. Asset identity also includes native asset type. Workspace subtype, names, and email do not identify an object.</x:v>
       </x:c>
       <x:c r="C13" s="17" t="str">
         <x:v>Registry reconciliation</x:v>
@@ -946,7 +946,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R37cb9a51087c417a"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R954f0b7a33f440d6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1020,7 +1020,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re348627782404da5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ae71ea844534097"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1112,7 +1112,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ref01c47526934f4d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ca802527de84404"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1204,7 +1204,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re7a5777105a948f2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8a006110e91f4a54"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1278,7 +1278,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R169aecea494e415e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R433f4badf717405f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1397,7 +1397,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbccb69c61b1c4f44"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfe42702ea1b2426a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1775,7 +1775,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -1792,10 +1792,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -2312,7 +2312,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="F37" s="17" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="G37" s="17" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -3364,7 +3364,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R52e780e0296d4a40"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R40c4eaf2650b48f8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3742,7 +3742,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -3759,10 +3759,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -5331,7 +5331,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra74472e52ad94676"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3dcfee9fb89f486d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -5709,7 +5709,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="17" ht="36" customHeight="1">
+    <x:row r="17" ht="47.25" customHeight="1">
       <x:c r="A17" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -5726,10 +5726,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="F17" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="G17" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="H17" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -7298,7 +7298,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcfecaf919c8f4108"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6cd10b1c7670438b"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8569,7 +8569,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="39" ht="47.25" customHeight="1">
+    <x:row r="39" ht="58.5" customHeight="1">
       <x:c r="A39" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8583,7 +8583,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E39" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F39" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -8595,16 +8595,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I39" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J39" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K39" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="40" ht="47.25" customHeight="1">
+    <x:row r="40" ht="58.5" customHeight="1">
       <x:c r="A40" s="4" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8618,7 +8618,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E40" s="4" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F40" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -8630,16 +8630,16 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I40" s="4" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J40" s="4" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K40" s="4" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
       </x:c>
     </x:row>
-    <x:row r="41" ht="47.25" customHeight="1">
+    <x:row r="41" ht="58.5" customHeight="1">
       <x:c r="A41" s="17" t="str">
         <x:v>Coverage</x:v>
       </x:c>
@@ -8653,7 +8653,7 @@
         <x:v>Conditional</x:v>
       </x:c>
       <x:c r="E41" s="17" t="str">
-        <x:v>Number of delivered data rows, excluding header and fully blank template rows. Complete requires a count; zero is valid only for a verified empty collection.</x:v>
+        <x:v>Exact number of delivered rows, excluding headers and fully blank template rows. Complete and Partial require a nonnegative count, including zero. Failed and NotCollected require NULL and no data rows. Count alone does not prove scope completeness.</x:v>
       </x:c>
       <x:c r="F41" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -8665,10 +8665,10 @@
         <x:v>Count from the completed export</x:v>
       </x:c>
       <x:c r="I41" s="17" t="str">
-        <x:v>Nonnegative delivered row count. Complete requires an exact count, including a legitimate zero. Failed/NotCollected use NULL.</x:v>
+        <x:v>Complete and Partial require the exact nonnegative delivered row count. Zero is valid. Failed and NotCollected require NULL and no dataset rows. Only independently verified complete scope supports absence comparisons.</x:v>
       </x:c>
       <x:c r="J41" s="17" t="str">
-        <x:v>NULL when absent from this export. NULL means unknown, not false or not applicable.</x:v>
+        <x:v>NULL only for Failed or NotCollected. A missing count blocks a Complete or Partial delivery.</x:v>
       </x:c>
       <x:c r="K41" s="17" t="str">
         <x:v>https://github.com/dlpate2525/analytic-registry/tree/main/platform-data-collection/v1.1-extract</x:v>
@@ -10459,7 +10459,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="93" ht="47.25" customHeight="1">
+    <x:row r="93" ht="58.5" customHeight="1">
       <x:c r="A93" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10473,7 +10473,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E93" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F93" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10494,7 +10494,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="94" ht="47.25" customHeight="1">
+    <x:row r="94" ht="58.5" customHeight="1">
       <x:c r="A94" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10508,7 +10508,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E94" s="4" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F94" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10529,7 +10529,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="95" ht="47.25" customHeight="1">
+    <x:row r="95" ht="58.5" customHeight="1">
       <x:c r="A95" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10543,7 +10543,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E95" s="17" t="str">
-        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Alteryx V1 does not collect connections. Missing or unstable keys require review.</x:v>
+        <x:v>Tableau data connection LUID or returned Power BI source-instance ID. Resolves a Connection RegistryObject within its platform, instance, and native scope. Alteryx V1.1 does not collect connections. Names and endpoint details do not identify this object.</x:v>
       </x:c>
       <x:c r="F95" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10578,7 +10578,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E96" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F96" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10613,7 +10613,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E97" s="17" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F97" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10648,7 +10648,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E98" s="4" t="str">
-        <x:v>Source caption when available. The Power BI adapter uses an explicit technology-and-ID label when no supported name is provided. Maps to ObservedConnection.DisplayName.</x:v>
+        <x:v>Source caption when available. The Power BI adapter uses a technology-and-ID label when no supported name is provided. Maps to ObjectObservation.DisplayName, never the business name.</x:v>
       </x:c>
       <x:c r="F98" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10669,7 +10669,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="99" ht="47.25" customHeight="1">
+    <x:row r="99" ht="58.5" customHeight="1">
       <x:c r="A99" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10683,7 +10683,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E99" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F99" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10704,7 +10704,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="100" ht="47.25" customHeight="1">
+    <x:row r="100" ht="58.5" customHeight="1">
       <x:c r="A100" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10718,7 +10718,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E100" s="4" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F100" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10730,7 +10730,7 @@
         <x:v>public.data_connections.dbclass</x:v>
       </x:c>
       <x:c r="I100" s="4" t="str">
-        <x:v>Map oracle to Oracle, sqlserver to SQL Server, dataengine/hyper to Extract; retain other known values or Undefined.</x:v>
+        <x:v>Map oracle to Oracle and sqlserver to SQL Server. Preserve other native dbclass values, including dataengine and hyper. Use Undefined only when missing; HasExtract is independent.</x:v>
       </x:c>
       <x:c r="J100" s="4" t="str">
         <x:v>Reject or quarantine a nonblank row if missing. Never substitute a display name.</x:v>
@@ -10739,7 +10739,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="101" ht="47.25" customHeight="1">
+    <x:row r="101" ht="58.5" customHeight="1">
       <x:c r="A101" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10753,7 +10753,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E101" s="17" t="str">
-        <x:v>Source technology, such as Oracle or SQL Server. Null source types become Undefined. Preserve other vendor values for mapping review. Maps to resolved DataSource.TechnologyCode.</x:v>
+        <x:v>Source technology, such as Oracle or SQL Server. Missing source types become Undefined. Preserve other vendor values, including dataengine and hyper. Maps to ObjectObservation.TechnologyCode. HasExtract records extract evidence separately.</x:v>
       </x:c>
       <x:c r="F101" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10774,7 +10774,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="102" ht="47.25" customHeight="1">
+    <x:row r="102" ht="58.5" customHeight="1">
       <x:c r="A102" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10788,7 +10788,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E102" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F102" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -10809,7 +10809,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="103" ht="47.25" customHeight="1">
+    <x:row r="103" ht="58.5" customHeight="1">
       <x:c r="A103" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10823,7 +10823,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E103" s="17" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F103" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -10844,7 +10844,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="104" ht="47.25" customHeight="1">
+    <x:row r="104" ht="58.5" customHeight="1">
       <x:c r="A104" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10858,7 +10858,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E104" s="4" t="str">
-        <x:v>Tableau extract indicator, separate from source technology. Retained in staging. Power BI leaves it null; Alteryx V1 returns no connection rows.</x:v>
+        <x:v>Tableau extract indicator, independent from source technology. Maps to ObjectObservation.HasExtract with its value state. Preserve explicit true and false. Power BI leaves it null; Alteryx V1.1 returns no connection rows.</x:v>
       </x:c>
       <x:c r="F104" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -10893,7 +10893,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E105" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F105" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -10914,7 +10914,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="106" ht="36" customHeight="1">
+    <x:row r="106" ht="47.25" customHeight="1">
       <x:c r="A106" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -10928,7 +10928,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E106" s="4" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F106" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -10963,7 +10963,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E107" s="17" t="str">
-        <x:v>Allowed endpoint host from the source. Maps to DataSource.ServerHostname after endpoint resolution. Do not merge by host alone.</x:v>
+        <x:v>Allowed endpoint host from the source. Maps to ObjectObservation.ServerHostname on this connection. Do not merge connection identities by host or infer a shared cross-platform data source.</x:v>
       </x:c>
       <x:c r="F107" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -10998,7 +10998,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E108" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F108" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11019,7 +11019,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="109" ht="36" customHeight="1">
+    <x:row r="109" ht="47.25" customHeight="1">
       <x:c r="A109" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11033,7 +11033,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E109" s="17" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F109" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11068,7 +11068,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E110" s="4" t="str">
-        <x:v>Source database or provider-specific database identifier. Maps to DataSource.DatabaseName after validation.</x:v>
+        <x:v>Source database or provider-specific database identifier. Maps to ObjectObservation.DatabaseName on this connection. Shared data-source records and cross-platform endpoint matching are deferred.</x:v>
       </x:c>
       <x:c r="F110" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11103,7 +11103,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E111" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F111" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11138,7 +11138,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E112" s="4" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F112" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11173,7 +11173,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E113" s="17" t="str">
-        <x:v>Tableau native authentication method when present. Maps to ObservedConnection.AuthenticationTypeCode after vocabulary validation. Missing does not imply anonymous access.</x:v>
+        <x:v>Tableau native authentication method when present. Maps to ObjectObservation.AuthenticationTypeCode. Preserve the source code for mapping review. Missing does not imply anonymous access.</x:v>
       </x:c>
       <x:c r="F113" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -11208,7 +11208,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E114" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F114" s="4" t="str">
         <x:v>PowerBI</x:v>
@@ -11243,7 +11243,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E115" s="17" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F115" s="17" t="str">
         <x:v>Tableau</x:v>
@@ -11278,7 +11278,7 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="E116" s="4" t="str">
-        <x:v>Unknown for this pass. Maps to ObservedConnection.IdentityClassificationCode. Later identity evidence may support a service/personal classification.</x:v>
+        <x:v>Unknown for this pass. Maps to ObjectObservation.IdentityClassificationCode. Later verified identity evidence may establish a service or personal classification.</x:v>
       </x:c>
       <x:c r="F116" s="4" t="str">
         <x:v>Alteryx</x:v>
@@ -11299,7 +11299,7 @@
         <x:v>https://help.alteryx.com/20251/en/server/configure/database-management/mongodb-management/mongodb-schema-reference/alteryxgallery-mongodb-schema.html</x:v>
       </x:c>
     </x:row>
-    <x:row r="117" ht="47.25" customHeight="1">
+    <x:row r="117" ht="58.5" customHeight="1">
       <x:c r="A117" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11313,7 +11313,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E117" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F117" s="17" t="str">
         <x:v>PowerBI</x:v>
@@ -11334,7 +11334,7 @@
         <x:v>https://github.com/dlpate2525/analytic-registry/blob/main/platform-data-collection/v1.1-extract/fabric-query-mapping.md</x:v>
       </x:c>
     </x:row>
-    <x:row r="118" ht="36" customHeight="1">
+    <x:row r="118" ht="58.5" customHeight="1">
       <x:c r="A118" s="4" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11348,7 +11348,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E118" s="4" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F118" s="4" t="str">
         <x:v>Tableau</x:v>
@@ -11369,7 +11369,7 @@
         <x:v>https://tableau.github.io/tableau-data-dictionary/2026.2/data_dictionary.htm</x:v>
       </x:c>
     </x:row>
-    <x:row r="119" ht="47.25" customHeight="1">
+    <x:row r="119" ht="58.5" customHeight="1">
       <x:c r="A119" s="17" t="str">
         <x:v>Connections</x:v>
       </x:c>
@@ -11383,7 +11383,7 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="E119" s="17" t="str">
-        <x:v>Observed for the row's captured facts. Maps to ObservedConnection.EvidenceStatusCode. Dataset coverage controls what absences can mean.</x:v>
+        <x:v>Evidence for captured connection facts. Maps to ObjectObservation.EvidenceStatusCode. This projection reports Partial while credential controls remain unverified. Dataset coverage separately controls what absences can mean.</x:v>
       </x:c>
       <x:c r="F119" s="17" t="str">
         <x:v>Alteryx</x:v>
@@ -14977,7 +14977,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R43cdb629fb8b4ec6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra61eb6225581410c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17037,7 +17037,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R8817cb2ed65d4e28"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R25994da914184e96"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17138,7 +17138,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1e3746545f64e64"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd747f99e6db44827"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17203,7 +17203,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra62ab524e8fe4b35"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3812b6e9e2dd4ab2"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17277,7 +17277,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5fcd376d7e9549ad"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0a230eabe98481d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17360,7 +17360,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79abd5f8fde34660"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf07e43b6624348aa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17434,7 +17434,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5f2201369cc244a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3daffe014da44b38"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -17553,7 +17553,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1eddcdc3d1d845b1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c208403f7ee4d58"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>